<commit_message>
[20260412] Push fin de semana
</commit_message>
<xml_diff>
--- a/05_EXAMENES/preguntas_opcion_multiple_v2.xlsx
+++ b/05_EXAMENES/preguntas_opcion_multiple_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jorgejuvenalcamposferreira/Documents/GitHub/TC2001B.601-Ciencia-de-datos-ene-jun-2026/05_EXAMENES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B431F3-A743-424B-8445-F2FC4B354301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69497C8-73C8-D64D-8699-E9457F229E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="68800" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="607">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="953">
   <si>
     <t>tema</t>
   </si>
@@ -1171,21 +1171,6 @@
     <t>Los códigos hex #RRGGBB describen la intensidad de rojo, verde y azul en hexadecimal.</t>
   </si>
   <si>
-    <t>72 dpi</t>
-  </si>
-  <si>
-    <t>300 dpi</t>
-  </si>
-  <si>
-    <t>150 dpi</t>
-  </si>
-  <si>
-    <t>500 dpi</t>
-  </si>
-  <si>
-    <t>300 dpi es el estándar para impresión de alta calidad; 72 dpi basta para la web.</t>
-  </si>
-  <si>
     <t>Si llamamos ggsave("out.png") sin especificar el argumento plot, ¿qué gráfico se guarda?</t>
   </si>
   <si>
@@ -1414,9 +1399,6 @@
     <t>! invierte el valor lógico: !TRUE es FALSE y viceversa.</t>
   </si>
   <si>
-    <t>¿Cuál es la sintaxis correcta para definir una función propia en R?</t>
-  </si>
-  <si>
     <t>mi_funcion &lt;- function(x) { x^2 }</t>
   </si>
   <si>
@@ -1834,13 +1816,1069 @@
     <t>¿En qué se diferencian geom_col() y geom_bar() en ggplot2? (Buscar que hace geom_bar)</t>
   </si>
   <si>
-    <t xml:space="preserve">¿Qué resolución en DPI es recomendable al exportar gráficos con ggsave() para impresión? (Revisar, no visto en clase). </t>
-  </si>
-  <si>
     <t>Missing Completely At Random</t>
   </si>
   <si>
     <t>¿Por qué se considera al RCT (ensayo aleatorizado) el 'gold standard' o "estándar de oro" de la inferencia causal?</t>
+  </si>
+  <si>
+    <t>¿Qué operador se usa típicamente para asignar variables en R?</t>
+  </si>
+  <si>
+    <t>La asignación estándar en R se hace con el operador &lt;-.</t>
+  </si>
+  <si>
+    <t>¿Qué función se usa para crear un vector en R?</t>
+  </si>
+  <si>
+    <t>vec()</t>
+  </si>
+  <si>
+    <t>array()</t>
+  </si>
+  <si>
+    <t>La función c() concatena valores para formar vectores.</t>
+  </si>
+  <si>
+    <t>¿Qué función devuelve la raíz cuadrada de un número?</t>
+  </si>
+  <si>
+    <t>log()</t>
+  </si>
+  <si>
+    <t>abs()</t>
+  </si>
+  <si>
+    <t>round()</t>
+  </si>
+  <si>
+    <t>sqrt()</t>
+  </si>
+  <si>
+    <t>sqrt() calcula la raíz cuadrada.</t>
+  </si>
+  <si>
+    <t>¿Qué función obtiene el valor absoluto?</t>
+  </si>
+  <si>
+    <t>sd()</t>
+  </si>
+  <si>
+    <t>mean()</t>
+  </si>
+  <si>
+    <t>sum()</t>
+  </si>
+  <si>
+    <t>abs() devuelve el valor absoluto de un número.</t>
+  </si>
+  <si>
+    <t>Datos duplicados</t>
+  </si>
+  <si>
+    <t>Algoritmos de ML</t>
+  </si>
+  <si>
+    <t>Datos sobre los datos</t>
+  </si>
+  <si>
+    <t>Errores de medición</t>
+  </si>
+  <si>
+    <t>Los metadatos describen y contextualizan otros datos.</t>
+  </si>
+  <si>
+    <t>¿Qué nivel de la escalera analítica responde la pregunta '¿qué pasó?'</t>
+  </si>
+  <si>
+    <t>Cognitiva</t>
+  </si>
+  <si>
+    <t>Prescriptiva</t>
+  </si>
+  <si>
+    <t>Predictiva</t>
+  </si>
+  <si>
+    <t>Descriptiva</t>
+  </si>
+  <si>
+    <t>La analítica descriptiva explica lo que ocurrió.</t>
+  </si>
+  <si>
+    <t>¿Qué nivel de la escalera analítica responde '¿qué se debería hacer?'</t>
+  </si>
+  <si>
+    <t>Diagnóstica</t>
+  </si>
+  <si>
+    <t>La analítica prescriptiva recomienda acciones.</t>
+  </si>
+  <si>
+    <t>¿Qué tipo de análisis busca explicar por qué pasó algo?</t>
+  </si>
+  <si>
+    <t>Monitorización</t>
+  </si>
+  <si>
+    <t>Causalidad/diagnóstico</t>
+  </si>
+  <si>
+    <t>Descriptivo</t>
+  </si>
+  <si>
+    <t>Prescriptivo</t>
+  </si>
+  <si>
+    <t>El análisis de causalidad (diagnóstico) busca explicar causas.</t>
+  </si>
+  <si>
+    <t>¿Cuál es el primer paso del ciclo de trabajo con datos de Wickham?</t>
+  </si>
+  <si>
+    <t>Comunicar</t>
+  </si>
+  <si>
+    <t>Visualizar</t>
+  </si>
+  <si>
+    <t>Modelar</t>
+  </si>
+  <si>
+    <t>Importar</t>
+  </si>
+  <si>
+    <t>El ciclo inicia con la importación de datos.</t>
+  </si>
+  <si>
+    <t>¿Por qué es importante aprender a programar en ciencia de datos?</t>
+  </si>
+  <si>
+    <t>Para evitar el análisis de datos</t>
+  </si>
+  <si>
+    <t>Para automatizar, reproducir y escalar análisis</t>
+  </si>
+  <si>
+    <t>Para trabajar sin datos</t>
+  </si>
+  <si>
+    <t>Solo para diseñar gráficos</t>
+  </si>
+  <si>
+    <t>La programación permite automatización, reproducibilidad y escalabilidad.</t>
+  </si>
+  <si>
+    <t>¿Qué es el directorio de trabajo en R?</t>
+  </si>
+  <si>
+    <t>La biblioteca de paquetes</t>
+  </si>
+  <si>
+    <t>La memoria RAM</t>
+  </si>
+  <si>
+    <t>El historial de comandos</t>
+  </si>
+  <si>
+    <t>La carpeta donde R busca y guarda archivos</t>
+  </si>
+  <si>
+    <t>El directorio de trabajo es la ruta por defecto para archivos.</t>
+  </si>
+  <si>
+    <t>¿Cuál es la ventaja principal de usar rutas relativas?</t>
+  </si>
+  <si>
+    <t>Mejoran la replicabilidad del código y facilitan a R el encontrar los archivos con los que trabaja</t>
+  </si>
+  <si>
+    <t>Mejora el funcionamiento de R en Mac, aunque no funciona tan bien en windows</t>
+  </si>
+  <si>
+    <t>Son más específicas que las rutas absolutas para la localización de archivos</t>
+  </si>
+  <si>
+    <t>Organizan automáticamente los archivos y el código en carpetas</t>
+  </si>
+  <si>
+    <t>Las rutas relativas hacen que el proyecto sea portátil.</t>
+  </si>
+  <si>
+    <t>¿Qué archivo establece el directorio de trabajo automáticamente en RStudio?</t>
+  </si>
+  <si>
+    <t>Un archivo .rds</t>
+  </si>
+  <si>
+    <t>Un archivo .RData</t>
+  </si>
+  <si>
+    <t>Un archivo .csv</t>
+  </si>
+  <si>
+    <t>Un archivo .Rproj</t>
+  </si>
+  <si>
+    <t>El archivo de proyecto .Rproj fija el directorio.</t>
+  </si>
+  <si>
+    <t>¿Cuál es la estructura recomendada en clase para un proyecto de R?</t>
+  </si>
+  <si>
+    <t>Carpetas Data, Script y Output</t>
+  </si>
+  <si>
+    <t>Carpetas Temp y Cache solamente</t>
+  </si>
+  <si>
+    <t>Solo una carpeta con todo</t>
+  </si>
+  <si>
+    <t>Carpetas Logs y Bin</t>
+  </si>
+  <si>
+    <t>Se sugiere separar datos, scripts y resultados.</t>
+  </si>
+  <si>
+    <t>¿Qué paquete se usó en clase para leer archivos Excel?</t>
+  </si>
+  <si>
+    <t>readxl proporciona read_excel() para Excel.</t>
+  </si>
+  <si>
+    <t>¿Qué paquete se usó en clase para leer archivos Stata .dta?</t>
+  </si>
+  <si>
+    <t>ggthemes</t>
+  </si>
+  <si>
+    <t>stringr</t>
+  </si>
+  <si>
+    <t>plotly</t>
+  </si>
+  <si>
+    <t>haven incluye read_dta() para Stata.</t>
+  </si>
+  <si>
+    <t>¿Qué es el tidyverse?</t>
+  </si>
+  <si>
+    <t>Una filosofía de programación que no tiene nada que ver con código</t>
+  </si>
+  <si>
+    <t>Colección de paquetes con filosofía común</t>
+  </si>
+  <si>
+    <t>Un solo paquete para bases de datos</t>
+  </si>
+  <si>
+    <t>Un lenguaje distinto a R</t>
+  </si>
+  <si>
+    <t>El tidyverse integra paquetes con una gramática común.</t>
+  </si>
+  <si>
+    <t>¿Para que sirve el operador pipe %&gt;% en tidyverse?</t>
+  </si>
+  <si>
+    <t>Concatenar funciones como 'y después', y pasar el resultado de lo que hay detrás del operador como el primer argumento de la siguiente función</t>
+  </si>
+  <si>
+    <t>Multiplicar matrices</t>
+  </si>
+  <si>
+    <t>Multiplicar vectores</t>
+  </si>
+  <si>
+    <t>Ordenar columnas</t>
+  </si>
+  <si>
+    <t>El pipe pasa el resultado a la siguiente función.</t>
+  </si>
+  <si>
+    <t>¿Cuál es la diferencia entre filter() y select()?</t>
+  </si>
+  <si>
+    <t>filter() elige columnas y select() filas</t>
+  </si>
+  <si>
+    <t>filter() resume y select() filtra</t>
+  </si>
+  <si>
+    <t>filter() ordena y select() agrupa</t>
+  </si>
+  <si>
+    <t>filter() elige filas y select() columnas</t>
+  </si>
+  <si>
+    <t>filter() conserva filas según condiciones; select() elige columnas.</t>
+  </si>
+  <si>
+    <t>¿Qué hace mutate() en dplyr?</t>
+  </si>
+  <si>
+    <t>Transforma o muta las tablas</t>
+  </si>
+  <si>
+    <t>Elimina columnas</t>
+  </si>
+  <si>
+    <t>Crea o modifica columnas</t>
+  </si>
+  <si>
+    <t>Ordena filas</t>
+  </si>
+  <si>
+    <t>mutate() agrega o transforma variables.</t>
+  </si>
+  <si>
+    <t>¿Para qué se usa group_by() junto con summarise()?</t>
+  </si>
+  <si>
+    <t>Para generar múltiples tablas a partir de grupos</t>
+  </si>
+  <si>
+    <t>Para obtener resúmenes o cálculos por grupo</t>
+  </si>
+  <si>
+    <t>Para crear gráficos</t>
+  </si>
+  <si>
+    <t>Para barajear las tablas y ordenar sus valores por grupos</t>
+  </si>
+  <si>
+    <t>group_by() agrupa y summarise() calcula estadísticas por grupo.</t>
+  </si>
+  <si>
+    <t>¿Qué operador lógico representa AND en R?</t>
+  </si>
+  <si>
+    <t>&amp; combina condiciones con AND.</t>
+  </si>
+  <si>
+    <t>¿Qué geometría de ggplot2 se usa para un scatter plot?</t>
+  </si>
+  <si>
+    <t>geom_histogram()</t>
+  </si>
+  <si>
+    <t>geom_point()</t>
+  </si>
+  <si>
+    <t>geom_boxplot()</t>
+  </si>
+  <si>
+    <t>geom_bar()</t>
+  </si>
+  <si>
+    <t>geom_point() crea gráficos de dispersión.</t>
+  </si>
+  <si>
+    <t>¿Qué función se usa para guardar una gráfica en archivo de imagen?</t>
+  </si>
+  <si>
+    <t>write.csv()</t>
+  </si>
+  <si>
+    <t>saveRDS()</t>
+  </si>
+  <si>
+    <t>ggsave() exporta gráficos de ggplot2.</t>
+  </si>
+  <si>
+    <t>¿Qué hace left_join() en dplyr?</t>
+  </si>
+  <si>
+    <t>Conserva todas las filas de una tabla izquierda y le une los datos de una tabla derecha</t>
+  </si>
+  <si>
+    <t>Conserva solo coincidencias perfectas</t>
+  </si>
+  <si>
+    <t>Conserva los datos de las tablas izquierda y derecha, rellenando las no coincidencias con valores Nas</t>
+  </si>
+  <si>
+    <t>Conserva todas las filas de una tabla derecha y le une los datos de una tabla izquierda</t>
+  </si>
+  <si>
+    <t>left_join() mantiene todas las filas de la tabla izquierda.</t>
+  </si>
+  <si>
+    <t>¿Qué hace inner_join()?</t>
+  </si>
+  <si>
+    <t>Conserva todas las filas de la tabla derecha</t>
+  </si>
+  <si>
+    <t>Combina columnas de una sola tabla</t>
+  </si>
+  <si>
+    <t>Devuelve solo filas con coincidencia en ambas tablas</t>
+  </si>
+  <si>
+    <t>Devuelve filas sin coincidencia</t>
+  </si>
+  <si>
+    <t>inner_join() conserva solo coincidencias.</t>
+  </si>
+  <si>
+    <t>¿Qué hace pivot_longer()?</t>
+  </si>
+  <si>
+    <t>Convierte una tabla de formato largo a formato ancho</t>
+  </si>
+  <si>
+    <t>Ordena alfabéticamente</t>
+  </si>
+  <si>
+    <t>Elimina valores NA</t>
+  </si>
+  <si>
+    <t>Convierte una tabla de formato ancho a formato largo</t>
+  </si>
+  <si>
+    <t>pivot_longer() reestructura columnas a filas.</t>
+  </si>
+  <si>
+    <t>¿Cómo ordenarías de mayor a menor una variable con dplyr?</t>
+  </si>
+  <si>
+    <t>arrange(desc(variable)) o arrange(-variable)</t>
+  </si>
+  <si>
+    <t>sort(variable)</t>
+  </si>
+  <si>
+    <t>arrange(asc(variable)) o arrange(variable)</t>
+  </si>
+  <si>
+    <t>reorder(variable)</t>
+  </si>
+  <si>
+    <t>desc() ordena en forma descendente.</t>
+  </si>
+  <si>
+    <t>En un join entre empleo estatal y grado promedio de educación estatal, ¿qué columna común, de las siguientes, recomendaría usar como variable llave?</t>
+  </si>
+  <si>
+    <t>tasa_desempleo</t>
+  </si>
+  <si>
+    <t>edad</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>cve_ent</t>
+  </si>
+  <si>
+    <t>La llave compartida es cve_ent.</t>
+  </si>
+  <si>
+    <t>¿Qué función convierte una tabla de formato ancho (wide) a formato largo (long)?</t>
+  </si>
+  <si>
+    <t>separate()</t>
+  </si>
+  <si>
+    <t>unite()</t>
+  </si>
+  <si>
+    <t>pivot_longer() transforma columnas en filas.</t>
+  </si>
+  <si>
+    <t>¿Cómo se crea un factor ordenado en R?</t>
+  </si>
+  <si>
+    <t>str_c(x)</t>
+  </si>
+  <si>
+    <t>factor(x, levels = c(...))</t>
+  </si>
+  <si>
+    <t>as.Date(x)</t>
+  </si>
+  <si>
+    <t>factor()</t>
+  </si>
+  <si>
+    <t>factor() con levels define el orden de categorías.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Qué función personaliza manualmente los colores en los elementos gráficos de ggplot2? Esto es, que a cada categoría de la gráfica le podemos asignar un color específico.(Ojo, no el fill, sino el color). </t>
+  </si>
+  <si>
+    <t>scale_color_brewer()</t>
+  </si>
+  <si>
+    <t>scale_color_manual()</t>
+  </si>
+  <si>
+    <t>scale_color_gradientn()</t>
+  </si>
+  <si>
+    <t>theme_minimal()</t>
+  </si>
+  <si>
+    <t>scale_color_manual() define paletas específicas.</t>
+  </si>
+  <si>
+    <t>¿Qué geometría se usa para barras con valores ya calculados?</t>
+  </si>
+  <si>
+    <t>geom_line()</t>
+  </si>
+  <si>
+    <t>geom_col()</t>
+  </si>
+  <si>
+    <t>geom_col() usa valores existentes en el eje y.</t>
+  </si>
+  <si>
+    <t>¿Qué geom agrega etiquetas de texto a una gráfica?</t>
+  </si>
+  <si>
+    <t>geom_bin2d()</t>
+  </si>
+  <si>
+    <t>geom_density()</t>
+  </si>
+  <si>
+    <t>geom_smooth()</t>
+  </si>
+  <si>
+    <t>geom_text() añade etiquetas a los puntos/barras.</t>
+  </si>
+  <si>
+    <t>¿Qué hace theme_minimal() en ggplot2?</t>
+  </si>
+  <si>
+    <t>Elimina datos NA</t>
+  </si>
+  <si>
+    <t>Agrupa variables</t>
+  </si>
+  <si>
+    <t>Aplica un tema visual minimalista</t>
+  </si>
+  <si>
+    <t>Cambia el sistema de coordenadas</t>
+  </si>
+  <si>
+    <t>theme_minimal() ajusta el estilo de la gráfica.</t>
+  </si>
+  <si>
+    <t>¿Cuál de estos es un componente de ggplot2?</t>
+  </si>
+  <si>
+    <t>install.packages()</t>
+  </si>
+  <si>
+    <t>geom_*()</t>
+  </si>
+  <si>
+    <t>Las geometrías geom_* son capas esenciales de ggplot2.</t>
+  </si>
+  <si>
+    <t>¿Qué hace aes() en ggplot2?</t>
+  </si>
+  <si>
+    <t>Define el tipo de geometría a utilizar</t>
+  </si>
+  <si>
+    <t>Guarda la gráfica</t>
+  </si>
+  <si>
+    <t>Elimina outliers</t>
+  </si>
+  <si>
+    <t>Mapea variables a elementos estéticos de la gráfica</t>
+  </si>
+  <si>
+    <t>aes() conecta variables con propiedades visuales.</t>
+  </si>
+  <si>
+    <t>¿Cuál es la diferencia entre asignar color dentro vs. fuera de aes()?</t>
+  </si>
+  <si>
+    <t>Fuera crea facetas</t>
+  </si>
+  <si>
+    <t>Dentro elimina leyenda</t>
+  </si>
+  <si>
+    <t>Dentro mapea una variable; fuera fija un color</t>
+  </si>
+  <si>
+    <t>Dentro de aes() crea un mapeo por variable.</t>
+  </si>
+  <si>
+    <t>¿Qué capa de ggplot controla el sistema de coordenadas?</t>
+  </si>
+  <si>
+    <t>coord_*()</t>
+  </si>
+  <si>
+    <t>theme_*()</t>
+  </si>
+  <si>
+    <t>scale_*()</t>
+  </si>
+  <si>
+    <t>facet_*()</t>
+  </si>
+  <si>
+    <t>coord_*() define el sistema de coordenadas.</t>
+  </si>
+  <si>
+    <t>¿Qué capa de ggplot se usa para dividir la gráfica en paneles?</t>
+  </si>
+  <si>
+    <t>stat_*()</t>
+  </si>
+  <si>
+    <t>facet_*() crea facetas por categorías.</t>
+  </si>
+  <si>
+    <t>¿Qué capa de ggplot define el estilo visual general?</t>
+  </si>
+  <si>
+    <t>aes()</t>
+  </si>
+  <si>
+    <t>theme_*() ajusta tipografías, fondos y grillas.</t>
+  </si>
+  <si>
+    <t>¿Qué es la carga cognitiva en visualización?</t>
+  </si>
+  <si>
+    <t>El esfuerzo mental requerido para procesar la gráfica</t>
+  </si>
+  <si>
+    <t>El tamaño del archivo</t>
+  </si>
+  <si>
+    <t>El número de columnas</t>
+  </si>
+  <si>
+    <t>La resolución de la pantalla</t>
+  </si>
+  <si>
+    <t>La carga cognitiva describe el esfuerzo mental del usuario.</t>
+  </si>
+  <si>
+    <t>¿Qué hace facet_wrap() en ggplot2?</t>
+  </si>
+  <si>
+    <t>Convierte a formato largo</t>
+  </si>
+  <si>
+    <t>Crea una cuadrícula por una variable categórica</t>
+  </si>
+  <si>
+    <t>Elimina leyendas</t>
+  </si>
+  <si>
+    <t>Agrega una línea de tendencia</t>
+  </si>
+  <si>
+    <t>facet_wrap() separa la gráfica por categorías.</t>
+  </si>
+  <si>
+    <t>¿Qué significa scales = 'free_y' en facet_wrap()?</t>
+  </si>
+  <si>
+    <t>Elimina el eje Y</t>
+  </si>
+  <si>
+    <t>Todas las facetas comparten la misma escala</t>
+  </si>
+  <si>
+    <t>Cada faceta tiene su propia escala en Y</t>
+  </si>
+  <si>
+    <t>Convierte a logaritmo</t>
+  </si>
+  <si>
+    <t>free_y permite que cada panel ajuste su rango.</t>
+  </si>
+  <si>
+    <t>¿Cómo se define una función personalizada en R?</t>
+  </si>
+  <si>
+    <t>nombre_funcion &lt;- func() { ... }</t>
+  </si>
+  <si>
+    <t>nombre_funcion &lt;- def() { ... }</t>
+  </si>
+  <si>
+    <t>nombre_funcion &lt;- lambda() { ... }</t>
+  </si>
+  <si>
+    <t>nombre_funcion &lt;- function() { ... }</t>
+  </si>
+  <si>
+    <t>En R las funciones se crean con function().</t>
+  </si>
+  <si>
+    <t>¿Cuándo es preferible usar la mediana en lugar de la media?</t>
+  </si>
+  <si>
+    <t>Cuando hay muchos ceros</t>
+  </si>
+  <si>
+    <t>Cuando la distribución de una variable es insesgada</t>
+  </si>
+  <si>
+    <t>Cuando hay outliers o distribuciones sesgadas</t>
+  </si>
+  <si>
+    <t>Cuando los datos están perfectamente normales</t>
+  </si>
+  <si>
+    <t>La mediana es robusta a valores extremos.</t>
+  </si>
+  <si>
+    <t>¿Cómo se define la varianza?</t>
+  </si>
+  <si>
+    <t>Como una forma de definir que tan dispersos están los datos</t>
+  </si>
+  <si>
+    <t>Como el promedio de desviaciones cuadráticas respecto a la media</t>
+  </si>
+  <si>
+    <t>Como el valor máximo menos el valor mínimo (rango)</t>
+  </si>
+  <si>
+    <t>Como la suma de todos los valores dividido entre el numero de valores que hay</t>
+  </si>
+  <si>
+    <t>La varianza mide dispersión alrededor de la media.</t>
+  </si>
+  <si>
+    <t>¿Qué relación hay entre varianza y desviación estándar?</t>
+  </si>
+  <si>
+    <t>La opción B y la opción C son correctas en todos los casos</t>
+  </si>
+  <si>
+    <t>La desviación estándar es la raíz de la varianza</t>
+  </si>
+  <si>
+    <t>La varianza es la raíz de la desviación estándar</t>
+  </si>
+  <si>
+    <t>No están relacionadas</t>
+  </si>
+  <si>
+    <t>SD = sqrt(varianza).</t>
+  </si>
+  <si>
+    <t>¿Cómo se calcula el IQR (rango intercuantílico)?</t>
+  </si>
+  <si>
+    <t>Q2 - Q1</t>
+  </si>
+  <si>
+    <t>Max - Min</t>
+  </si>
+  <si>
+    <t>Q4 - Q2</t>
+  </si>
+  <si>
+    <t>Q3 - Q1</t>
+  </si>
+  <si>
+    <t>El rango intercuartílico es Q3 menos Q1.</t>
+  </si>
+  <si>
+    <t>¿Qué regla se usa para detectar outliers con IQR?</t>
+  </si>
+  <si>
+    <t>Valores fuera de media ± 1 deviación estándar</t>
+  </si>
+  <si>
+    <t>Valores por debajo de Q1 o por encima de Q3</t>
+  </si>
+  <si>
+    <t>Valores por encima o por debajo de ± 1.96*IQR</t>
+  </si>
+  <si>
+    <t>Valores por debajo de Q1 - 1.5*IQR o por encima de Q3 + 1.5*IQR</t>
+  </si>
+  <si>
+    <t>La regla de 1.5*IQR detecta valores extremos.</t>
+  </si>
+  <si>
+    <t>¿Qué significa MCAR en datos faltantes?</t>
+  </si>
+  <si>
+    <t>Missing Conditionally At Risk</t>
+  </si>
+  <si>
+    <t>Missing Causally At Random</t>
+  </si>
+  <si>
+    <t>Missing Centrally At Random</t>
+  </si>
+  <si>
+    <t>MCAR indica ausencia completamente aleatoria.</t>
+  </si>
+  <si>
+    <t>¿Qué plantea el modelo causal de Rubin?</t>
+  </si>
+  <si>
+    <t>Modelo clásico de machine learning para obtener la causalidad de un evento</t>
+  </si>
+  <si>
+    <t>Resultados potenciales Y(1) y Y(0) y efecto causal definido como Y(1) - Y(0)</t>
+  </si>
+  <si>
+    <t>Modelo de clustering</t>
+  </si>
+  <si>
+    <t>Método de imputación de valores faltantes a partir de una explicación causal Y(1)</t>
+  </si>
+  <si>
+    <t>El modelo de Rubin usa resultados potenciales.</t>
+  </si>
+  <si>
+    <t>¿Qué es un confundidor (confounder)?</t>
+  </si>
+  <si>
+    <t>Variable que afecta tratamiento y resultado</t>
+  </si>
+  <si>
+    <t>Variable irrelevante</t>
+  </si>
+  <si>
+    <t>Variable que solo afecta el resultado</t>
+  </si>
+  <si>
+    <t>Variable aleatoria</t>
+  </si>
+  <si>
+    <t>Un confundidor afecta tanto la causa como el efecto.</t>
+  </si>
+  <si>
+    <t>¿Cuál es el estimador básico de Diferencias en Diferencias?</t>
+  </si>
+  <si>
+    <t>Suma de residuos</t>
+  </si>
+  <si>
+    <t>Coeficiente de correlación</t>
+  </si>
+  <si>
+    <t>(Post-Treated - Pre-Treated) - (Post-Control - Pre-Control)</t>
+  </si>
+  <si>
+    <t>Media tratada menos media control</t>
+  </si>
+  <si>
+    <t>DiD compara cambios antes y después entre grupos.</t>
+  </si>
+  <si>
+    <t>¿Qué es una regresión discontinua (RD)?</t>
+  </si>
+  <si>
+    <t>Un modelo de series de tiempo</t>
+  </si>
+  <si>
+    <t>Método que explota un umbral de asignación</t>
+  </si>
+  <si>
+    <t>Un modelo sin variables</t>
+  </si>
+  <si>
+    <t>RD usa discontinuidades en un cutoff para inferir causalidad.</t>
+  </si>
+  <si>
+    <t>¿Por qué correlación no implica causación?</t>
+  </si>
+  <si>
+    <t>Porque no hay datos suficientes</t>
+  </si>
+  <si>
+    <t>Porque es un error matemático</t>
+  </si>
+  <si>
+    <t>Porque siempre es cero cuando hay causalidad</t>
+  </si>
+  <si>
+    <t>Puede haber confusores o causalidad inversa</t>
+  </si>
+  <si>
+    <t>La correlación puede deberse a factores externos.</t>
+  </si>
+  <si>
+    <t>¿Qué función en R redondea un número?</t>
+  </si>
+  <si>
+    <t>round() redondea valores numéricos a decimales definidos.</t>
+  </si>
+  <si>
+    <t>¿Qué pregunta responde el análisis predictivo?</t>
+  </si>
+  <si>
+    <t>¿Qué pasó?</t>
+  </si>
+  <si>
+    <t>¿Qué pasará?</t>
+  </si>
+  <si>
+    <t>¿Por qué pasó?</t>
+  </si>
+  <si>
+    <t>¿Qué se debería hacer?</t>
+  </si>
+  <si>
+    <t>La analítica predictiva busca anticipar resultados futuros.</t>
+  </si>
+  <si>
+    <t>¿Qué etapa del ciclo de Wickham ocurre después de limpiar datos?</t>
+  </si>
+  <si>
+    <t>Transformar</t>
+  </si>
+  <si>
+    <t>El flujo es Importar → Limpiar → Transformar.</t>
+  </si>
+  <si>
+    <t>¿Qué hace arrange() en dplyr?</t>
+  </si>
+  <si>
+    <t>Filtra columnas</t>
+  </si>
+  <si>
+    <t>Ordena filas según una o más variables</t>
+  </si>
+  <si>
+    <t>Crea nuevas columnas</t>
+  </si>
+  <si>
+    <t>Agrupa datos</t>
+  </si>
+  <si>
+    <t>arrange() ordena filas en el dataframe.</t>
+  </si>
+  <si>
+    <t>¿Qué hace right_join()?</t>
+  </si>
+  <si>
+    <t>Devuelve filas no coincidentes</t>
+  </si>
+  <si>
+    <t>Solo filas coincidentes</t>
+  </si>
+  <si>
+    <t>Conserva todas las filas de la tabla izquierda</t>
+  </si>
+  <si>
+    <t>right_join() mantiene todas las filas de la tabla derecha.</t>
+  </si>
+  <si>
+    <t>¿Qué función convierte de formato largo a ancho?</t>
+  </si>
+  <si>
+    <t>pivot_wider() expande categorías a columnas.</t>
+  </si>
+  <si>
+    <t>¿Qué función se usa para concatenar strings en tidyverse?</t>
+  </si>
+  <si>
+    <t>as.character()</t>
+  </si>
+  <si>
+    <t>str_c()</t>
+  </si>
+  <si>
+    <t>toupper()</t>
+  </si>
+  <si>
+    <t>paste0()</t>
+  </si>
+  <si>
+    <t>str_c() de stringr concatena texto.</t>
+  </si>
+  <si>
+    <t>¿Qué hace clean_names() de janitor?</t>
+  </si>
+  <si>
+    <t>Estandariza nombres de columnas</t>
+  </si>
+  <si>
+    <t>Genera gráficos</t>
+  </si>
+  <si>
+    <t>Convierte a factor</t>
+  </si>
+  <si>
+    <t>Elimina filas duplicadas</t>
+  </si>
+  <si>
+    <t>clean_names() limpia y normaliza nombres de variables.</t>
+  </si>
+  <si>
+    <t>¿Para qué se usa write_xlsx() en R?</t>
+  </si>
+  <si>
+    <t>Generar HTML</t>
+  </si>
+  <si>
+    <t>Crear gráficos</t>
+  </si>
+  <si>
+    <t>Guardar archivos Excel</t>
+  </si>
+  <si>
+    <t>Leer archivos CSV</t>
+  </si>
+  <si>
+    <t>write_xlsx() exporta dataframes a Excel.</t>
+  </si>
+  <si>
+    <t>¿Qué gráfico es ideal para detectar outliers?</t>
+  </si>
+  <si>
+    <t>Gráfica de áreas</t>
+  </si>
+  <si>
+    <t>Mapa de calor</t>
+  </si>
+  <si>
+    <t>Gráfica de pastel</t>
+  </si>
+  <si>
+    <t>Boxplot</t>
+  </si>
+  <si>
+    <t>El boxplot muestra puntos extremos fuera del rango.</t>
+  </si>
+  <si>
+    <t>¿Qué es un contrafáctico o contrafactual?</t>
+  </si>
+  <si>
+    <t>Un dato faltante MCAR</t>
+  </si>
+  <si>
+    <t>Una variable instrumental</t>
+  </si>
+  <si>
+    <t>Un modelo predictivo</t>
+  </si>
+  <si>
+    <t>Resultado potencial no observado</t>
+  </si>
+  <si>
+    <t>El contrafáctico es el resultado que no se observa.</t>
+  </si>
+  <si>
+    <t>¿Cuál es la sintaxis correcta para definir una función propia en R? (En este caso, una función que eleve un número al cuadrado)</t>
   </si>
 </sst>
 </file>
@@ -1888,11 +2926,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2196,7 +3237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:H168"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2237,7 +3278,7 @@
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>598</v>
+        <v>592</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -2367,7 +3408,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>599</v>
+        <v>593</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>42</v>
@@ -2419,7 +3460,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>600</v>
+        <v>594</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>53</v>
@@ -2575,7 +3616,7 @@
         <v>68</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>602</v>
+        <v>596</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>87</v>
@@ -2587,7 +3628,7 @@
         <v>89</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>601</v>
+        <v>595</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>20</v>
@@ -3563,7 +4604,7 @@
         <v>287</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>603</v>
+        <v>597</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>306</v>
@@ -3901,25 +4942,25 @@
         <v>346</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>604</v>
+        <v>383</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="32" x14ac:dyDescent="0.2">
@@ -3927,25 +4968,25 @@
         <v>346</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="32" x14ac:dyDescent="0.2">
@@ -3953,192 +4994,192 @@
         <v>346</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
-        <v>346</v>
+        <v>401</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="C69" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="D69" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="G69" s="2" t="s">
+      <c r="B70" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="G70" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H69" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" ht="48" x14ac:dyDescent="0.2">
-      <c r="A70" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="H70" s="2" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
-        <v>406</v>
+        <v>432</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>439</v>
+        <v>9</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>440</v>
@@ -4150,7 +5191,7 @@
         <v>442</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>443</v>
@@ -4158,94 +5199,94 @@
     </row>
     <row r="76" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>444</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>9</v>
+        <v>445</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>451</v>
+        <v>298</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>452</v>
       </c>
       <c r="F77" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H77" s="2" t="s">
         <v>453</v>
-      </c>
-      <c r="G77" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H77" s="2" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B78" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C78" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="D78" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="E78" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="D78" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="E78" s="2" t="s">
+      <c r="F78" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="F78" s="2" t="s">
-        <v>446</v>
-      </c>
       <c r="G78" s="2" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B79" s="2" t="s">
+        <v>952</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>459</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="D79" s="2" t="s">
         <v>460</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>447</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>461</v>
@@ -4254,7 +5295,7 @@
         <v>462</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>463</v>
@@ -4262,7 +5303,7 @@
     </row>
     <row r="80" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>464</v>
@@ -4280,7 +5321,7 @@
         <v>468</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="H80" s="2" t="s">
         <v>469</v>
@@ -4288,7 +5329,7 @@
     </row>
     <row r="81" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>470</v>
@@ -4306,7 +5347,7 @@
         <v>474</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="H81" s="2" t="s">
         <v>475</v>
@@ -4314,7 +5355,7 @@
     </row>
     <row r="82" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>476</v>
@@ -4332,7 +5373,7 @@
         <v>480</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="H82" s="2" t="s">
         <v>481</v>
@@ -4340,33 +5381,33 @@
     </row>
     <row r="83" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
-        <v>437</v>
+        <v>482</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>489</v>
@@ -4384,7 +5425,7 @@
         <v>493</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="H84" s="2" t="s">
         <v>494</v>
@@ -4392,7 +5433,7 @@
     </row>
     <row r="85" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>495</v>
@@ -4410,7 +5451,7 @@
         <v>499</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="H85" s="2" t="s">
         <v>500</v>
@@ -4418,7 +5459,7 @@
     </row>
     <row r="86" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>501</v>
@@ -4436,7 +5477,7 @@
         <v>505</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>506</v>
@@ -4444,7 +5485,7 @@
     </row>
     <row r="87" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>507</v>
@@ -4462,7 +5503,7 @@
         <v>511</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="H87" s="2" t="s">
         <v>512</v>
@@ -4470,7 +5511,7 @@
     </row>
     <row r="88" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>513</v>
@@ -4488,7 +5529,7 @@
         <v>517</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="H88" s="2" t="s">
         <v>518</v>
@@ -4496,39 +5537,39 @@
     </row>
     <row r="89" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>519</v>
       </c>
       <c r="C89" s="2" t="s">
+        <v>598</v>
+      </c>
+      <c r="D89" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="D89" s="2" t="s">
+      <c r="E89" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="E89" s="2" t="s">
+      <c r="F89" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="F89" s="2" t="s">
+      <c r="G89" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H89" s="2" t="s">
         <v>523</v>
-      </c>
-      <c r="G89" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H89" s="2" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B90" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="C90" s="2" t="s">
         <v>525</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>605</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>526</v>
@@ -4540,7 +5581,7 @@
         <v>528</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="H90" s="2" t="s">
         <v>529</v>
@@ -4548,7 +5589,7 @@
     </row>
     <row r="91" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>530</v>
@@ -4566,7 +5607,7 @@
         <v>534</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="H91" s="2" t="s">
         <v>535</v>
@@ -4574,59 +5615,59 @@
     </row>
     <row r="92" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>536</v>
       </c>
       <c r="C92" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H92" s="2" t="s">
         <v>537</v>
       </c>
-      <c r="D92" s="2" t="s">
+    </row>
+    <row r="93" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A93" s="2" t="s">
         <v>538</v>
       </c>
-      <c r="E92" s="2" t="s">
+      <c r="B93" s="2" t="s">
         <v>539</v>
       </c>
-      <c r="F92" s="2" t="s">
+      <c r="C93" s="2" t="s">
         <v>540</v>
       </c>
-      <c r="G92" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H92" s="2" t="s">
+      <c r="D93" s="2" t="s">
         <v>541</v>
       </c>
-    </row>
-    <row r="93" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A93" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="B93" s="2" t="s">
+      <c r="E93" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="C93" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="E93" s="2" t="s">
-        <v>261</v>
-      </c>
       <c r="F93" s="2" t="s">
-        <v>260</v>
+        <v>543</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>545</v>
@@ -4644,15 +5685,15 @@
         <v>549</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>550</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>551</v>
@@ -4670,44 +5711,44 @@
         <v>555</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="H95" s="2" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B96" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="C96" s="2" t="s">
         <v>557</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="D96" s="2" t="s">
         <v>558</v>
       </c>
-      <c r="D96" s="2" t="s">
+      <c r="E96" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="E96" s="2" t="s">
+      <c r="F96" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="F96" s="2" t="s">
+      <c r="G96" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H96" s="2" t="s">
         <v>561</v>
-      </c>
-      <c r="G96" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H96" s="2" t="s">
-        <v>562</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>606</v>
+        <v>562</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>563</v>
@@ -4722,15 +5763,15 @@
         <v>566</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H97" s="2" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>568</v>
@@ -4748,15 +5789,15 @@
         <v>572</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H98" s="2" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>574</v>
@@ -4774,15 +5815,15 @@
         <v>578</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="H99" s="2" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>580</v>
@@ -4800,15 +5841,15 @@
         <v>584</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H100" s="2" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>586</v>
@@ -4826,36 +5867,1752 @@
         <v>590</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="H101" s="2" t="s">
         <v>591</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="48" x14ac:dyDescent="0.2">
-      <c r="A102" s="2" t="s">
-        <v>544</v>
-      </c>
-      <c r="B102" s="2" t="s">
-        <v>592</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>594</v>
-      </c>
-      <c r="E102" s="2" t="s">
-        <v>595</v>
-      </c>
-      <c r="F102" s="2" t="s">
-        <v>596</v>
-      </c>
-      <c r="G102" s="2" t="s">
+    <row r="102" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>8</v>
+      </c>
+      <c r="B102" t="s">
+        <v>600</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E102" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F102" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G102" t="s">
+        <v>20</v>
+      </c>
+      <c r="H102" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>8</v>
+      </c>
+      <c r="B103" t="s">
+        <v>602</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F103" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G103" t="s">
+        <v>20</v>
+      </c>
+      <c r="H103" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>8</v>
+      </c>
+      <c r="B104" t="s">
+        <v>606</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="F104" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="G104" t="s">
+        <v>20</v>
+      </c>
+      <c r="H104" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>8</v>
+      </c>
+      <c r="B105" t="s">
+        <v>612</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>613</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="G105" t="s">
+        <v>13</v>
+      </c>
+      <c r="H105" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>68</v>
+      </c>
+      <c r="B106" t="s">
+        <v>114</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>617</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="G106" t="s">
+        <v>13</v>
+      </c>
+      <c r="H106" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>68</v>
+      </c>
+      <c r="B107" t="s">
+        <v>622</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="G107" t="s">
+        <v>20</v>
+      </c>
+      <c r="H107" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>68</v>
+      </c>
+      <c r="B108" t="s">
+        <v>628</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="F108" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="G108" t="s">
+        <v>13</v>
+      </c>
+      <c r="H108" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>68</v>
+      </c>
+      <c r="B109" t="s">
+        <v>631</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>633</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="G109" t="s">
         <v>34</v>
       </c>
-      <c r="H102" s="2" t="s">
-        <v>597</v>
+      <c r="H109" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>68</v>
+      </c>
+      <c r="B110" t="s">
+        <v>637</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="E110" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="F110" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="G110" t="s">
+        <v>20</v>
+      </c>
+      <c r="H110" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>68</v>
+      </c>
+      <c r="B111" t="s">
+        <v>643</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="E111" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="F111" s="3" t="s">
+        <v>647</v>
+      </c>
+      <c r="G111" t="s">
+        <v>34</v>
+      </c>
+      <c r="H111" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>120</v>
+      </c>
+      <c r="B112" t="s">
+        <v>649</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="E112" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="G112" t="s">
+        <v>20</v>
+      </c>
+      <c r="H112" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>120</v>
+      </c>
+      <c r="B113" t="s">
+        <v>655</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="E113" s="3" t="s">
+        <v>658</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="G113" t="s">
+        <v>27</v>
+      </c>
+      <c r="H113" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>120</v>
+      </c>
+      <c r="B114" t="s">
+        <v>661</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>662</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>663</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="G114" t="s">
+        <v>20</v>
+      </c>
+      <c r="H114" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>120</v>
+      </c>
+      <c r="B115" t="s">
+        <v>667</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="E115" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>671</v>
+      </c>
+      <c r="G115" t="s">
+        <v>27</v>
+      </c>
+      <c r="H115" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>120</v>
+      </c>
+      <c r="B116" t="s">
+        <v>673</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="G116" t="s">
+        <v>27</v>
+      </c>
+      <c r="H116" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>120</v>
+      </c>
+      <c r="B117" t="s">
+        <v>675</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>676</v>
+      </c>
+      <c r="E117" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="F117" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="G117" t="s">
+        <v>27</v>
+      </c>
+      <c r="H117" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>175</v>
+      </c>
+      <c r="B118" t="s">
+        <v>680</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>681</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>682</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>683</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>684</v>
+      </c>
+      <c r="G118" t="s">
+        <v>34</v>
+      </c>
+      <c r="H118" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>175</v>
+      </c>
+      <c r="B119" t="s">
+        <v>686</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="E119" s="3" t="s">
+        <v>689</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="G119" t="s">
+        <v>27</v>
+      </c>
+      <c r="H119" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>175</v>
+      </c>
+      <c r="B120" t="s">
+        <v>692</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="G120" t="s">
+        <v>20</v>
+      </c>
+      <c r="H120" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>175</v>
+      </c>
+      <c r="B121" t="s">
+        <v>698</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>700</v>
+      </c>
+      <c r="E121" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>702</v>
+      </c>
+      <c r="G121" t="s">
+        <v>13</v>
+      </c>
+      <c r="H121" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>175</v>
+      </c>
+      <c r="B122" t="s">
+        <v>704</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="E122" s="3" t="s">
+        <v>707</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="G122" t="s">
+        <v>34</v>
+      </c>
+      <c r="H122" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>175</v>
+      </c>
+      <c r="B123" t="s">
+        <v>710</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="E123" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="F123" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="G123" t="s">
+        <v>27</v>
+      </c>
+      <c r="H123" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>175</v>
+      </c>
+      <c r="B124" t="s">
+        <v>712</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="E124" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="F124" s="3" t="s">
+        <v>716</v>
+      </c>
+      <c r="G124" t="s">
+        <v>34</v>
+      </c>
+      <c r="H124" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>175</v>
+      </c>
+      <c r="B125" t="s">
+        <v>718</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E125" s="3" t="s">
+        <v>719</v>
+      </c>
+      <c r="F125" s="3" t="s">
+        <v>720</v>
+      </c>
+      <c r="G125" t="s">
+        <v>27</v>
+      </c>
+      <c r="H125" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>231</v>
+      </c>
+      <c r="B126" t="s">
+        <v>722</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>724</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>725</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>726</v>
+      </c>
+      <c r="G126" t="s">
+        <v>27</v>
+      </c>
+      <c r="H126" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>231</v>
+      </c>
+      <c r="B127" t="s">
+        <v>728</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>729</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>730</v>
+      </c>
+      <c r="E127" s="3" t="s">
+        <v>731</v>
+      </c>
+      <c r="F127" s="3" t="s">
+        <v>732</v>
+      </c>
+      <c r="G127" t="s">
+        <v>13</v>
+      </c>
+      <c r="H127" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>231</v>
+      </c>
+      <c r="B128" t="s">
+        <v>734</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>735</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>737</v>
+      </c>
+      <c r="F128" s="3" t="s">
+        <v>738</v>
+      </c>
+      <c r="G128" t="s">
+        <v>20</v>
+      </c>
+      <c r="H128" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
+        <v>231</v>
+      </c>
+      <c r="B129" t="s">
+        <v>740</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>741</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>742</v>
+      </c>
+      <c r="E129" s="3" t="s">
+        <v>743</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>744</v>
+      </c>
+      <c r="G129" t="s">
+        <v>27</v>
+      </c>
+      <c r="H129" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
+        <v>231</v>
+      </c>
+      <c r="B130" t="s">
+        <v>746</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="E130" s="3" t="s">
+        <v>749</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="G130" t="s">
+        <v>20</v>
+      </c>
+      <c r="H130" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A131" t="s">
+        <v>287</v>
+      </c>
+      <c r="B131" t="s">
+        <v>752</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>753</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E131" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>754</v>
+      </c>
+      <c r="G131" t="s">
+        <v>13</v>
+      </c>
+      <c r="H131" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
+        <v>287</v>
+      </c>
+      <c r="B132" t="s">
+        <v>756</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>757</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>758</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>759</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="G132" t="s">
+        <v>34</v>
+      </c>
+      <c r="H132" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
+        <v>287</v>
+      </c>
+      <c r="B133" t="s">
+        <v>762</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="E133" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>766</v>
+      </c>
+      <c r="G133" t="s">
+        <v>34</v>
+      </c>
+      <c r="H133" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
+        <v>287</v>
+      </c>
+      <c r="B134" t="s">
+        <v>768</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>770</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>716</v>
+      </c>
+      <c r="G134" t="s">
+        <v>34</v>
+      </c>
+      <c r="H134" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A135" t="s">
+        <v>287</v>
+      </c>
+      <c r="B135" t="s">
+        <v>772</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="E135" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="F135" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="G135" t="s">
+        <v>20</v>
+      </c>
+      <c r="H135" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
+        <v>287</v>
+      </c>
+      <c r="B136" t="s">
+        <v>777</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="F136" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="G136" t="s">
+        <v>13</v>
+      </c>
+      <c r="H136" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A137" t="s">
+        <v>346</v>
+      </c>
+      <c r="B137" t="s">
+        <v>783</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E137" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="F137" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="G137" t="s">
+        <v>20</v>
+      </c>
+      <c r="H137" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
+        <v>346</v>
+      </c>
+      <c r="B138" t="s">
+        <v>787</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>789</v>
+      </c>
+      <c r="E138" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>791</v>
+      </c>
+      <c r="G138" t="s">
+        <v>20</v>
+      </c>
+      <c r="H138" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A139" t="s">
+        <v>346</v>
+      </c>
+      <c r="B139" t="s">
+        <v>793</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="E139" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="G139" t="s">
+        <v>20</v>
+      </c>
+      <c r="H139" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
+        <v>346</v>
+      </c>
+      <c r="B140" t="s">
+        <v>798</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>800</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>801</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="G140" t="s">
+        <v>27</v>
+      </c>
+      <c r="H140" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
+        <v>346</v>
+      </c>
+      <c r="B141" t="s">
+        <v>804</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="E141" s="3" t="s">
+        <v>800</v>
+      </c>
+      <c r="F141" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="G141" t="s">
+        <v>34</v>
+      </c>
+      <c r="H141" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A142" t="s">
+        <v>346</v>
+      </c>
+      <c r="B142" t="s">
+        <v>807</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>800</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="E142" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="F142" s="3" t="s">
+        <v>808</v>
+      </c>
+      <c r="G142" t="s">
+        <v>27</v>
+      </c>
+      <c r="H142" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
+        <v>401</v>
+      </c>
+      <c r="B143" t="s">
+        <v>810</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>812</v>
+      </c>
+      <c r="E143" s="3" t="s">
+        <v>813</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="G143" t="s">
+        <v>27</v>
+      </c>
+      <c r="H143" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
+        <v>432</v>
+      </c>
+      <c r="B144" t="s">
+        <v>816</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>817</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="E144" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>820</v>
+      </c>
+      <c r="G144" t="s">
+        <v>34</v>
+      </c>
+      <c r="H144" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
+        <v>432</v>
+      </c>
+      <c r="B145" t="s">
+        <v>822</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>823</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>824</v>
+      </c>
+      <c r="E145" s="3" t="s">
+        <v>825</v>
+      </c>
+      <c r="F145" s="3" t="s">
+        <v>826</v>
+      </c>
+      <c r="G145" t="s">
+        <v>13</v>
+      </c>
+      <c r="H145" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
+        <v>432</v>
+      </c>
+      <c r="B146" t="s">
+        <v>828</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>829</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>830</v>
+      </c>
+      <c r="E146" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="F146" s="3" t="s">
+        <v>832</v>
+      </c>
+      <c r="G146" t="s">
+        <v>20</v>
+      </c>
+      <c r="H146" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A147" t="s">
+        <v>482</v>
+      </c>
+      <c r="B147" t="s">
+        <v>834</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>836</v>
+      </c>
+      <c r="E147" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>838</v>
+      </c>
+      <c r="G147" t="s">
+        <v>13</v>
+      </c>
+      <c r="H147" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A148" t="s">
+        <v>482</v>
+      </c>
+      <c r="B148" t="s">
+        <v>840</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>841</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>842</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="G148" t="s">
+        <v>34</v>
+      </c>
+      <c r="H148" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A149" t="s">
+        <v>482</v>
+      </c>
+      <c r="B149" t="s">
+        <v>846</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>847</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>848</v>
+      </c>
+      <c r="E149" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="F149" s="3" t="s">
+        <v>850</v>
+      </c>
+      <c r="G149" t="s">
+        <v>34</v>
+      </c>
+      <c r="H149" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A150" t="s">
+        <v>482</v>
+      </c>
+      <c r="B150" t="s">
+        <v>852</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>854</v>
+      </c>
+      <c r="E150" s="3" t="s">
+        <v>855</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="G150" t="s">
+        <v>20</v>
+      </c>
+      <c r="H150" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
+        <v>482</v>
+      </c>
+      <c r="B151" t="s">
+        <v>858</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>859</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>860</v>
+      </c>
+      <c r="E151" s="3" t="s">
+        <v>861</v>
+      </c>
+      <c r="F151" s="3" t="s">
+        <v>862</v>
+      </c>
+      <c r="G151" t="s">
+        <v>20</v>
+      </c>
+      <c r="H151" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
+        <v>482</v>
+      </c>
+      <c r="B152" t="s">
+        <v>864</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="E152" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="F152" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="G152" t="s">
+        <v>27</v>
+      </c>
+      <c r="H152" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A153" t="s">
+        <v>538</v>
+      </c>
+      <c r="B153" t="s">
+        <v>869</v>
+      </c>
+      <c r="C153" s="3" t="s">
+        <v>870</v>
+      </c>
+      <c r="D153" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="E153" s="3" t="s">
+        <v>872</v>
+      </c>
+      <c r="F153" s="3" t="s">
+        <v>873</v>
+      </c>
+      <c r="G153" t="s">
+        <v>34</v>
+      </c>
+      <c r="H153" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A154" t="s">
+        <v>538</v>
+      </c>
+      <c r="B154" t="s">
+        <v>875</v>
+      </c>
+      <c r="C154" s="3" t="s">
+        <v>876</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="E154" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="F154" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="G154" t="s">
+        <v>27</v>
+      </c>
+      <c r="H154" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A155" t="s">
+        <v>538</v>
+      </c>
+      <c r="B155" t="s">
+        <v>881</v>
+      </c>
+      <c r="C155" s="3" t="s">
+        <v>882</v>
+      </c>
+      <c r="D155" s="3" t="s">
+        <v>883</v>
+      </c>
+      <c r="E155" s="3" t="s">
+        <v>884</v>
+      </c>
+      <c r="F155" s="3" t="s">
+        <v>885</v>
+      </c>
+      <c r="G155" t="s">
+        <v>13</v>
+      </c>
+      <c r="H155" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A156" t="s">
+        <v>538</v>
+      </c>
+      <c r="B156" t="s">
+        <v>887</v>
+      </c>
+      <c r="C156" s="3" t="s">
+        <v>888</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E156" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="F156" s="3" t="s">
+        <v>890</v>
+      </c>
+      <c r="G156" t="s">
+        <v>13</v>
+      </c>
+      <c r="H156" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A157" t="s">
+        <v>538</v>
+      </c>
+      <c r="B157" t="s">
+        <v>892</v>
+      </c>
+      <c r="C157" s="3" t="s">
+        <v>893</v>
+      </c>
+      <c r="D157" s="3" t="s">
+        <v>894</v>
+      </c>
+      <c r="E157" s="3" t="s">
+        <v>895</v>
+      </c>
+      <c r="F157" s="3" t="s">
+        <v>896</v>
+      </c>
+      <c r="G157" t="s">
+        <v>20</v>
+      </c>
+      <c r="H157" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A158" t="s">
+        <v>8</v>
+      </c>
+      <c r="B158" t="s">
+        <v>898</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="D158" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="E158" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="G158" t="s">
+        <v>13</v>
+      </c>
+      <c r="H158" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A159" t="s">
+        <v>68</v>
+      </c>
+      <c r="B159" t="s">
+        <v>900</v>
+      </c>
+      <c r="C159" s="3" t="s">
+        <v>901</v>
+      </c>
+      <c r="D159" s="3" t="s">
+        <v>902</v>
+      </c>
+      <c r="E159" s="3" t="s">
+        <v>903</v>
+      </c>
+      <c r="F159" s="3" t="s">
+        <v>904</v>
+      </c>
+      <c r="G159" t="s">
+        <v>34</v>
+      </c>
+      <c r="H159" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A160" t="s">
+        <v>68</v>
+      </c>
+      <c r="B160" t="s">
+        <v>906</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="E160" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="F160" s="3" t="s">
+        <v>907</v>
+      </c>
+      <c r="G160" t="s">
+        <v>20</v>
+      </c>
+      <c r="H160" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A161" t="s">
+        <v>175</v>
+      </c>
+      <c r="B161" t="s">
+        <v>909</v>
+      </c>
+      <c r="C161" s="3" t="s">
+        <v>910</v>
+      </c>
+      <c r="D161" s="3" t="s">
+        <v>911</v>
+      </c>
+      <c r="E161" s="3" t="s">
+        <v>912</v>
+      </c>
+      <c r="F161" s="3" t="s">
+        <v>913</v>
+      </c>
+      <c r="G161" t="s">
+        <v>34</v>
+      </c>
+      <c r="H161" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A162" t="s">
+        <v>231</v>
+      </c>
+      <c r="B162" t="s">
+        <v>915</v>
+      </c>
+      <c r="C162" s="3" t="s">
+        <v>916</v>
+      </c>
+      <c r="D162" s="3" t="s">
+        <v>917</v>
+      </c>
+      <c r="E162" s="3" t="s">
+        <v>918</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>729</v>
+      </c>
+      <c r="G162" t="s">
+        <v>20</v>
+      </c>
+      <c r="H162" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A163" t="s">
+        <v>231</v>
+      </c>
+      <c r="B163" t="s">
+        <v>920</v>
+      </c>
+      <c r="C163" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D163" s="3" t="s">
+        <v>753</v>
+      </c>
+      <c r="E163" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="F163" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="G163" t="s">
+        <v>13</v>
+      </c>
+      <c r="H163" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A164" t="s">
+        <v>287</v>
+      </c>
+      <c r="B164" t="s">
+        <v>922</v>
+      </c>
+      <c r="C164" s="3" t="s">
+        <v>923</v>
+      </c>
+      <c r="D164" s="3" t="s">
+        <v>924</v>
+      </c>
+      <c r="E164" s="3" t="s">
+        <v>925</v>
+      </c>
+      <c r="F164" s="3" t="s">
+        <v>926</v>
+      </c>
+      <c r="G164" t="s">
+        <v>34</v>
+      </c>
+      <c r="H164" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A165" t="s">
+        <v>287</v>
+      </c>
+      <c r="B165" t="s">
+        <v>928</v>
+      </c>
+      <c r="C165" s="3" t="s">
+        <v>929</v>
+      </c>
+      <c r="D165" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="E165" s="3" t="s">
+        <v>931</v>
+      </c>
+      <c r="F165" s="3" t="s">
+        <v>932</v>
+      </c>
+      <c r="G165" t="s">
+        <v>27</v>
+      </c>
+      <c r="H165" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A166" t="s">
+        <v>432</v>
+      </c>
+      <c r="B166" t="s">
+        <v>934</v>
+      </c>
+      <c r="C166" s="3" t="s">
+        <v>935</v>
+      </c>
+      <c r="D166" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="E166" s="3" t="s">
+        <v>937</v>
+      </c>
+      <c r="F166" s="3" t="s">
+        <v>938</v>
+      </c>
+      <c r="G166" t="s">
+        <v>13</v>
+      </c>
+      <c r="H166" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A167" t="s">
+        <v>482</v>
+      </c>
+      <c r="B167" t="s">
+        <v>940</v>
+      </c>
+      <c r="C167" s="3" t="s">
+        <v>941</v>
+      </c>
+      <c r="D167" s="3" t="s">
+        <v>942</v>
+      </c>
+      <c r="E167" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="F167" s="3" t="s">
+        <v>944</v>
+      </c>
+      <c r="G167" t="s">
+        <v>20</v>
+      </c>
+      <c r="H167" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A168" t="s">
+        <v>538</v>
+      </c>
+      <c r="B168" t="s">
+        <v>946</v>
+      </c>
+      <c r="C168" s="3" t="s">
+        <v>947</v>
+      </c>
+      <c r="D168" s="3" t="s">
+        <v>948</v>
+      </c>
+      <c r="E168" s="3" t="s">
+        <v>949</v>
+      </c>
+      <c r="F168" s="3" t="s">
+        <v>950</v>
+      </c>
+      <c r="G168" t="s">
+        <v>20</v>
+      </c>
+      <c r="H168" t="s">
+        <v>951</v>
       </c>
     </row>
   </sheetData>

</xml_diff>